<commit_message>
Add GitHub Actions workflow for scheduled daily runs
</commit_message>
<xml_diff>
--- a/reports/summary_2026-06-25.xlsx
+++ b/reports/summary_2026-06-25.xlsx
@@ -446,20 +446,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BillAckman</t>
+          <t>aleabitoreddit</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>12210</v>
+        <v>10091</v>
       </c>
       <c r="D2" t="n">
-        <v>1372</v>
+        <v>693</v>
       </c>
       <c r="E2" t="n">
-        <v>4070</v>
+        <v>1261.4</v>
       </c>
     </row>
     <row r="3">
@@ -469,35 +469,35 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" t="n">
-        <v>10847</v>
+        <v>9109</v>
       </c>
       <c r="D3" t="n">
-        <v>895</v>
+        <v>864</v>
       </c>
       <c r="E3" t="n">
-        <v>570.9</v>
+        <v>506.1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>aleabitoreddit</t>
+          <t>BillAckman</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>9043</v>
+        <v>3719</v>
       </c>
       <c r="D4" t="n">
-        <v>580</v>
+        <v>421</v>
       </c>
       <c r="E4" t="n">
-        <v>1130.4</v>
+        <v>1859.5</v>
       </c>
     </row>
     <row r="5">
@@ -510,13 +510,13 @@
         <v>7</v>
       </c>
       <c r="C5" t="n">
-        <v>1509</v>
+        <v>1645</v>
       </c>
       <c r="D5" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="E5" t="n">
-        <v>215.6</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6">
@@ -526,92 +526,92 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C6" t="n">
-        <v>332</v>
+        <v>198</v>
       </c>
       <c r="D6" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E6" t="n">
-        <v>30.2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>xingpt</t>
+          <t>bboczeng</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C7" t="n">
-        <v>132</v>
+        <v>104</v>
       </c>
       <c r="D7" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>33</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>bboczeng</t>
+          <t>DariusDale42</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E8" t="n">
-        <v>9.6</v>
+        <v>33.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DariusDale42</t>
+          <t>dnystedt</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E9" t="n">
-        <v>31</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>dnystedt</t>
+          <t>xingpt</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>11.5</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Yahoo Finance market data integration and Elon Musk to watchlist
</commit_message>
<xml_diff>
--- a/reports/summary_2026-06-25.xlsx
+++ b/reports/summary_2026-06-25.xlsx
@@ -453,13 +453,13 @@
         <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>10091</v>
+        <v>12728</v>
       </c>
       <c r="D2" t="n">
-        <v>693</v>
+        <v>889</v>
       </c>
       <c r="E2" t="n">
-        <v>1261.4</v>
+        <v>1591</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C3" t="n">
-        <v>9109</v>
+        <v>8939</v>
       </c>
       <c r="D3" t="n">
-        <v>864</v>
+        <v>672</v>
       </c>
       <c r="E3" t="n">
-        <v>506.1</v>
+        <v>470.5</v>
       </c>
     </row>
     <row r="4">
@@ -491,13 +491,13 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>3719</v>
+        <v>4471</v>
       </c>
       <c r="D4" t="n">
-        <v>421</v>
+        <v>496</v>
       </c>
       <c r="E4" t="n">
-        <v>1859.5</v>
+        <v>2235.5</v>
       </c>
     </row>
     <row r="5">
@@ -507,54 +507,54 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>1645</v>
+        <v>1706</v>
       </c>
       <c r="D5" t="n">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E5" t="n">
-        <v>235</v>
+        <v>189.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tengyanAI</t>
+          <t>bboczeng</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C6" t="n">
-        <v>198</v>
+        <v>375</v>
       </c>
       <c r="D6" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E6" t="n">
-        <v>22</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>bboczeng</t>
+          <t>tengyanAI</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C7" t="n">
-        <v>104</v>
+        <v>215</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="E7" t="n">
-        <v>13</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="8">
@@ -564,16 +564,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C8" t="n">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>33.7</v>
+        <v>28.8</v>
       </c>
     </row>
     <row r="9">
@@ -586,13 +586,13 @@
         <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="D9" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9" t="n">
-        <v>19.8</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="10">
@@ -602,16 +602,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C10" t="n">
-        <v>24</v>
+        <v>94</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E10" t="n">
-        <v>8</v>
+        <v>13.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>